<commit_message>
Upgrade Meta API and disable creative recommendations
</commit_message>
<xml_diff>
--- a/template/ads template.xlsx
+++ b/template/ads template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <r>
       <rPr>
@@ -83,10 +83,10 @@
     <t xml:space="preserve">{$header_description_2}</t>
   </si>
   <si>
-    <t xml:space="preserve">Warszawa – Test - {$campain_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.25</t>
+    <t xml:space="preserve">url_address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warszawa – Test – address -  {$campain_date}</t>
   </si>
   <si>
     <t xml:space="preserve">52.22876759117127</t>
@@ -113,64 +113,7 @@
     <t xml:space="preserve">header description Warszawa 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Katowice – Test - {$campain_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50.26720611348598</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19.030295909543366</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w Katowicach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pozdrawiam Katowice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header Katowice 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header Katowice 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header description Katowice 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header description Katowice 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandomierz – Test - {$campain_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50.68250925592705</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.752933193364505</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w Sandomierzu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pozdrawiam Sandomierz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header Sandomierz 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header Sandomierz 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header description Sandomierz 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header description Sandomierz 2</t>
+    <t xml:space="preserve">https://malygeniusz.org/</t>
   </si>
 </sst>
 </file>
@@ -181,7 +124,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="d/mm/yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -232,6 +175,13 @@
       <color rgb="FF000000"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="238"/>
     </font>
   </fonts>
@@ -277,7 +227,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -299,6 +249,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -425,7 +379,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.2"/>
@@ -438,6 +392,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="27.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="33.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="27.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="23.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="15.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="25.04"/>
   </cols>
@@ -485,16 +440,19 @@
       <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>45430</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>15</v>
+        <v>46160</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>16</v>
@@ -506,10 +464,10 @@
         <v>13</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>45428</v>
+        <v>46158</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>45433</v>
+        <v>46163</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>18</v>
@@ -529,96 +487,14 @@
       <c r="N2" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="O2" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>45430</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>45432</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>45494</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>45430</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>45416</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>45556</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="O2" r:id="rId1" display="https://malygeniusz.org/"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>